<commit_message>
add test case in Excel sheet(article and search)
</commit_message>
<xml_diff>
--- a/wikipedia-Testing-ExcelSheet.xlsx
+++ b/wikipedia-Testing-ExcelSheet.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CODING\Devops\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECT\wikipedia_testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{4BF30EFE-FADD-463C-83B1-42B5A7EFEB8C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{98749B71-E0EC-41C3-A458-CBCADB68E3E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{23CE8EF5-60A8-44F8-8BB4-9FD29C3B8C6A}"/>
   </bookViews>
@@ -247,18 +247,9 @@
   </cellStyleXfs>
   <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -272,8 +263,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -603,86 +603,86 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
-      <c r="F1" s="7"/>
-      <c r="G1" s="7"/>
-      <c r="H1" s="7"/>
+      <c r="B1" s="4"/>
+      <c r="C1" s="4"/>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+      <c r="F1" s="4"/>
+      <c r="G1" s="4"/>
+      <c r="H1" s="4"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="6"/>
-      <c r="B2" s="7"/>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="7"/>
-      <c r="G2" s="7"/>
-      <c r="H2" s="7"/>
+      <c r="A2" s="3"/>
+      <c r="B2" s="4"/>
+      <c r="C2" s="4"/>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+      <c r="F2" s="4"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="7"/>
-      <c r="B3" s="7"/>
-      <c r="C3" s="7"/>
-      <c r="D3" s="7"/>
-      <c r="E3" s="7"/>
-      <c r="F3" s="7"/>
-      <c r="G3" s="7"/>
-      <c r="H3" s="7"/>
+      <c r="A3" s="4"/>
+      <c r="B3" s="4"/>
+      <c r="C3" s="4"/>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+      <c r="F3" s="4"/>
+      <c r="G3" s="4"/>
+      <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="8" t="s">
+      <c r="A4" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="7"/>
-      <c r="C4" s="9" t="s">
+      <c r="B4" s="4"/>
+      <c r="C4" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
-      <c r="F4" s="7" t="s">
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+      <c r="F4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="7"/>
-      <c r="H4" s="7"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="7"/>
-      <c r="B5" s="7"/>
-      <c r="C5" s="7"/>
-      <c r="D5" s="7"/>
-      <c r="E5" s="7"/>
-      <c r="F5" s="7"/>
-      <c r="G5" s="7"/>
-      <c r="H5" s="7"/>
+      <c r="A5" s="4"/>
+      <c r="B5" s="4"/>
+      <c r="C5" s="4"/>
+      <c r="D5" s="4"/>
+      <c r="E5" s="4"/>
+      <c r="F5" s="4"/>
+      <c r="G5" s="4"/>
+      <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A6" s="10" t="s">
+      <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="10" t="s">
+      <c r="D6" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="10" t="s">
+      <c r="E6" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="F6" s="10" t="s">
+      <c r="F6" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="10" t="s">
+      <c r="G6" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="H6" s="10" t="s">
+      <c r="H6" s="2" t="s">
         <v>14</v>
       </c>
     </row>
@@ -717,86 +717,86 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="5" t="s">
+      <c r="B4" s="8"/>
+      <c r="C4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1" t="s">
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
     </row>
     <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -830,86 +830,86 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="5" t="s">
+      <c r="B4" s="8"/>
+      <c r="C4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1" t="s">
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
     </row>
     <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="1" t="s">
         <v>5</v>
       </c>
     </row>
@@ -940,86 +940,86 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="2" t="s">
+      <c r="A1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="1"/>
-      <c r="C1" s="1"/>
-      <c r="D1" s="1"/>
-      <c r="E1" s="1"/>
-      <c r="F1" s="1"/>
-      <c r="G1" s="1"/>
-      <c r="H1" s="1"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="2"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-      <c r="F2" s="1"/>
-      <c r="G2" s="1"/>
-      <c r="H2" s="1"/>
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="1"/>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-      <c r="F3" s="1"/>
-      <c r="G3" s="1"/>
-      <c r="H3" s="1"/>
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="4" t="s">
+      <c r="A4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="1"/>
-      <c r="C4" s="5" t="s">
+      <c r="B4" s="8"/>
+      <c r="C4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="1"/>
-      <c r="E4" s="1"/>
-      <c r="F4" s="1" t="s">
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="1"/>
-      <c r="H4" s="1"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="1"/>
-      <c r="B5" s="1"/>
-      <c r="C5" s="1"/>
-      <c r="D5" s="1"/>
-      <c r="E5" s="1"/>
-      <c r="F5" s="1"/>
-      <c r="G5" s="1"/>
-      <c r="H5" s="1"/>
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
     </row>
     <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.35">
-      <c r="A6" s="3" t="s">
+      <c r="A6" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="3" t="s">
+      <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="3" t="s">
+      <c r="C6" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="D6" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="3" t="s">
+      <c r="E6" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="F6" s="3" t="s">
+      <c r="F6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G6" s="3" t="s">
+      <c r="G6" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="H6" s="3" t="s">
+      <c r="H6" s="1" t="s">
         <v>5</v>
       </c>
     </row>

</xml_diff>

<commit_message>
merge akash into main
</commit_message>
<xml_diff>
--- a/wikipedia-Testing-ExcelSheet.xlsx
+++ b/wikipedia-Testing-ExcelSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECT\wikipedia_testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF46ECD5-5D98-4908-B4BC-D304479B327A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D038705E-A186-44E1-86AF-239036070716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{23CE8EF5-60A8-44F8-8BB4-9FD29C3B8C6A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="42">
   <si>
     <t>Test Area / Functionality</t>
   </si>
@@ -214,19 +214,59 @@
     <t>Article_Page_Test.java</t>
   </si>
   <si>
-    <t>Article Page</t>
-  </si>
-  <si>
-    <t>Check whether article page opens correctly</t>
-  </si>
-  <si>
-    <t>Open an article and check the article page</t>
+    <t>Check article title after opening an article</t>
+  </si>
+  <si>
+    <t>Search India and check whether the correct title is displayed</t>
+  </si>
+  <si>
+    <t>Table_of_Content_test.java</t>
+  </si>
+  <si>
+    <t>Table of Contents</t>
+  </si>
+  <si>
+    <t>Check whether Table of Contents is displayed</t>
+  </si>
+  <si>
+    <t>Check Table of Contents on India article</t>
+  </si>
+  <si>
+    <t>Table_of_Content_Geography_test.java</t>
+  </si>
+  <si>
+    <t>Check whether Table of Contents section link works</t>
+  </si>
+  <si>
+    <t>Click Geography from Table of Contents</t>
+  </si>
+  <si>
+    <t>only when Screen is maximize</t>
   </si>
   <si>
     <t>1. Open ChromeBrowser
 2. Go to Wikipedia
-3. Search Youtube
-4. Check Result</t>
+3. Search India
+4. Click on Search button
+5. Check status on chrome browser</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBroswer
+2. Maximize the screen
+3. Go to the wikiPedia
+4. Search India
+5. click on search button
+6. check table of content is visible or not</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBroswer
+2. Maximize the screen
+3. Go to the wikiPedia
+4. Search India
+5. click on search button
+6. check table of content is visible or not
+7. click on Geography
+8. verify is it Geography or not</t>
   </si>
 </sst>
 </file>
@@ -317,9 +357,6 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -344,14 +381,17 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -671,81 +711,81 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="11.33203125" customWidth="1"/>
-    <col min="2" max="2" width="21.44140625" customWidth="1"/>
-    <col min="3" max="3" width="27.88671875" customWidth="1"/>
+    <col min="2" max="2" width="15.44140625" customWidth="1"/>
+    <col min="3" max="3" width="20.44140625" customWidth="1"/>
     <col min="4" max="4" width="23.88671875" customWidth="1"/>
-    <col min="5" max="5" width="25" customWidth="1"/>
-    <col min="6" max="6" width="25.21875" customWidth="1"/>
-    <col min="7" max="7" width="26.6640625" customWidth="1"/>
+    <col min="5" max="5" width="24.44140625" customWidth="1"/>
+    <col min="6" max="6" width="33.6640625" customWidth="1"/>
+    <col min="7" max="7" width="20.6640625" customWidth="1"/>
     <col min="8" max="8" width="31.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="6"/>
-      <c r="C1" s="6"/>
-      <c r="D1" s="6"/>
-      <c r="E1" s="6"/>
-      <c r="F1" s="6"/>
-      <c r="G1" s="6"/>
-      <c r="H1" s="6"/>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="5"/>
+      <c r="E1" s="5"/>
+      <c r="F1" s="5"/>
+      <c r="G1" s="5"/>
+      <c r="H1" s="5"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="5"/>
-      <c r="B2" s="6"/>
-      <c r="C2" s="6"/>
-      <c r="D2" s="6"/>
-      <c r="E2" s="6"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="6"/>
-      <c r="H2" s="6"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="5"/>
+      <c r="C2" s="5"/>
+      <c r="D2" s="5"/>
+      <c r="E2" s="5"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="5"/>
+      <c r="H2" s="5"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="6"/>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
-      <c r="H3" s="6"/>
+      <c r="A3" s="5"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
+      <c r="H3" s="5"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="7" t="s">
+      <c r="A4" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="6"/>
-      <c r="C4" s="8" t="s">
+      <c r="B4" s="5"/>
+      <c r="C4" s="7" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
-      <c r="F4" s="6" t="s">
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
+      <c r="F4" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="6"/>
-      <c r="H4" s="6"/>
+      <c r="G4" s="5"/>
+      <c r="H4" s="5"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="6"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="6"/>
-      <c r="H5" s="6"/>
-    </row>
-    <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A5" s="5"/>
+      <c r="B5" s="5"/>
+      <c r="C5" s="5"/>
+      <c r="D5" s="5"/>
+      <c r="E5" s="5"/>
+      <c r="F5" s="5"/>
+      <c r="G5" s="5"/>
+      <c r="H5" s="5"/>
+    </row>
+    <row r="6" spans="1:8" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="15" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="2" t="s">
+      <c r="C6" s="15" t="s">
         <v>0</v>
       </c>
       <c r="D6" s="2" t="s">
@@ -764,383 +804,411 @@
         <v>14</v>
       </c>
     </row>
-    <row r="7" spans="1:8" ht="62.4" x14ac:dyDescent="0.3">
-      <c r="A7" s="13">
+    <row r="7" spans="1:8" ht="108" x14ac:dyDescent="0.3">
+      <c r="A7" s="12">
         <v>1</v>
       </c>
-      <c r="B7" s="14" t="s">
+      <c r="B7" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="14" t="s">
+      <c r="C7" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D7" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="D7" s="14" t="s">
+      <c r="E7" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="E7" s="14" t="s">
+      <c r="F7" s="13" t="s">
+        <v>39</v>
+      </c>
+      <c r="G7" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="162" x14ac:dyDescent="0.3">
+      <c r="A8" s="12">
+        <v>2</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>16</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="D8" s="12" t="s">
+        <v>18</v>
+      </c>
+      <c r="E8" s="12" t="s">
+        <v>19</v>
+      </c>
+      <c r="F8" s="13" t="s">
+        <v>26</v>
+      </c>
+      <c r="G8" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="H8" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="108" x14ac:dyDescent="0.3">
+      <c r="A9" s="12">
+        <v>3</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="12" t="s">
+        <v>24</v>
+      </c>
+      <c r="E9" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="F9" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="G9" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="H9" s="12" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="132" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="12"/>
+      <c r="B10" s="12" t="s">
         <v>31</v>
       </c>
-      <c r="F7" s="15" t="s">
+      <c r="C10" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="G7" s="13" t="s">
+      <c r="D10" s="12" t="s">
+        <v>33</v>
+      </c>
+      <c r="E10" s="12" t="s">
+        <v>34</v>
+      </c>
+      <c r="F10" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="G10" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="H7" s="13" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="A8" s="13">
-        <v>2</v>
-      </c>
-      <c r="B8" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="C8" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="D8" s="14" t="s">
-        <v>18</v>
-      </c>
-      <c r="E8" s="14" t="s">
-        <v>19</v>
-      </c>
-      <c r="F8" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="G8" s="13" t="s">
+      <c r="H10" s="12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="162" x14ac:dyDescent="0.3">
+      <c r="A11" s="12"/>
+      <c r="B11" s="12" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>32</v>
+      </c>
+      <c r="D11" s="12" t="s">
+        <v>36</v>
+      </c>
+      <c r="E11" s="12" t="s">
+        <v>37</v>
+      </c>
+      <c r="F11" s="13" t="s">
+        <v>41</v>
+      </c>
+      <c r="G11" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="13" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" ht="93.6" x14ac:dyDescent="0.3">
-      <c r="A9" s="13">
-        <v>3</v>
-      </c>
-      <c r="B9" s="14" t="s">
-        <v>22</v>
-      </c>
-      <c r="C9" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="F9" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="G9" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="H9" s="13" t="s">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" ht="110.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="3"/>
-      <c r="B10" s="3"/>
-      <c r="C10" s="4"/>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
-      <c r="F10" s="3"/>
-      <c r="G10" s="3"/>
-      <c r="H10" s="3"/>
-    </row>
-    <row r="11" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="3"/>
-      <c r="B11" s="3"/>
-      <c r="C11" s="3"/>
-      <c r="D11" s="3"/>
-      <c r="E11" s="3"/>
-      <c r="F11" s="3"/>
-      <c r="G11" s="3"/>
-      <c r="H11" s="3"/>
-    </row>
-    <row r="12" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="3"/>
-      <c r="B12" s="3"/>
-      <c r="C12" s="3"/>
-      <c r="D12" s="3"/>
-      <c r="E12" s="3"/>
-      <c r="F12" s="3"/>
-      <c r="G12" s="3"/>
-      <c r="H12" s="3"/>
-    </row>
-    <row r="13" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="3"/>
-      <c r="B13" s="3"/>
-      <c r="C13" s="3"/>
-      <c r="D13" s="3"/>
-      <c r="E13" s="3"/>
-      <c r="F13" s="3"/>
-      <c r="G13" s="3"/>
-      <c r="H13" s="3"/>
-    </row>
-    <row r="14" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="3"/>
-      <c r="B14" s="3"/>
-      <c r="C14" s="3"/>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-      <c r="G14" s="3"/>
-      <c r="H14" s="3"/>
-    </row>
-    <row r="15" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="3"/>
-      <c r="B15" s="3"/>
-      <c r="C15" s="3"/>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-      <c r="G15" s="3"/>
-      <c r="H15" s="3"/>
-    </row>
-    <row r="16" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A16" s="3"/>
-      <c r="B16" s="3"/>
-      <c r="C16" s="3"/>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-      <c r="G16" s="3"/>
-      <c r="H16" s="3"/>
-    </row>
-    <row r="17" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A17" s="3"/>
-      <c r="B17" s="3"/>
-      <c r="C17" s="3"/>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-      <c r="G17" s="3"/>
-      <c r="H17" s="3"/>
-    </row>
-    <row r="18" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A18" s="3"/>
-      <c r="B18" s="3"/>
-      <c r="C18" s="3"/>
-      <c r="D18" s="3"/>
-      <c r="E18" s="3"/>
-      <c r="F18" s="3"/>
-      <c r="G18" s="3"/>
-      <c r="H18" s="3"/>
-    </row>
-    <row r="19" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A19" s="3"/>
-      <c r="B19" s="3"/>
-      <c r="C19" s="3"/>
-      <c r="D19" s="3"/>
-      <c r="E19" s="3"/>
-      <c r="F19" s="3"/>
-      <c r="G19" s="3"/>
-      <c r="H19" s="3"/>
-    </row>
-    <row r="20" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A20" s="3"/>
-      <c r="B20" s="3"/>
-      <c r="C20" s="3"/>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-      <c r="G20" s="3"/>
-      <c r="H20" s="3"/>
-    </row>
-    <row r="21" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A21" s="3"/>
-      <c r="B21" s="3"/>
-      <c r="C21" s="3"/>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-      <c r="G21" s="3"/>
-      <c r="H21" s="3"/>
-    </row>
-    <row r="22" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A22" s="3"/>
-      <c r="B22" s="3"/>
-      <c r="C22" s="3"/>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="3"/>
-      <c r="H22" s="3"/>
-    </row>
-    <row r="23" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A23" s="3"/>
-      <c r="B23" s="3"/>
-      <c r="C23" s="3"/>
-      <c r="D23" s="3"/>
-      <c r="E23" s="3"/>
-      <c r="F23" s="3"/>
-      <c r="G23" s="3"/>
-      <c r="H23" s="3"/>
-    </row>
-    <row r="24" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A24" s="3"/>
-      <c r="B24" s="3"/>
-      <c r="C24" s="3"/>
-      <c r="D24" s="3"/>
-      <c r="E24" s="3"/>
-      <c r="F24" s="3"/>
-      <c r="G24" s="3"/>
-      <c r="H24" s="3"/>
-    </row>
-    <row r="25" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A25" s="3"/>
-      <c r="B25" s="3"/>
-      <c r="C25" s="3"/>
-      <c r="D25" s="3"/>
-      <c r="E25" s="3"/>
-      <c r="F25" s="3"/>
-      <c r="G25" s="3"/>
-      <c r="H25" s="3"/>
-    </row>
-    <row r="26" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A26" s="3"/>
-      <c r="B26" s="3"/>
-      <c r="C26" s="3"/>
-      <c r="D26" s="3"/>
-      <c r="E26" s="3"/>
-      <c r="F26" s="3"/>
-      <c r="G26" s="3"/>
-      <c r="H26" s="3"/>
-    </row>
-    <row r="27" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A27" s="3"/>
-      <c r="B27" s="3"/>
-      <c r="C27" s="3"/>
-      <c r="D27" s="3"/>
-      <c r="E27" s="3"/>
-      <c r="F27" s="3"/>
-      <c r="G27" s="3"/>
-      <c r="H27" s="3"/>
-    </row>
-    <row r="28" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A28" s="3"/>
-      <c r="B28" s="3"/>
-      <c r="C28" s="3"/>
-      <c r="D28" s="3"/>
-      <c r="E28" s="3"/>
-      <c r="F28" s="3"/>
-      <c r="G28" s="3"/>
-      <c r="H28" s="3"/>
-    </row>
-    <row r="29" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A29" s="3"/>
-      <c r="B29" s="3"/>
-      <c r="C29" s="3"/>
-      <c r="D29" s="3"/>
-      <c r="E29" s="3"/>
-      <c r="F29" s="3"/>
-      <c r="G29" s="3"/>
-      <c r="H29" s="3"/>
-    </row>
-    <row r="30" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A30" s="3"/>
-      <c r="B30" s="3"/>
-      <c r="C30" s="3"/>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
-      <c r="G30" s="3"/>
-      <c r="H30" s="3"/>
-    </row>
-    <row r="31" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A31" s="3"/>
-      <c r="B31" s="3"/>
-      <c r="C31" s="3"/>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-      <c r="G31" s="3"/>
-      <c r="H31" s="3"/>
-    </row>
-    <row r="32" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A32" s="3"/>
-      <c r="B32" s="3"/>
-      <c r="C32" s="3"/>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-      <c r="G32" s="3"/>
-      <c r="H32" s="3"/>
-    </row>
-    <row r="33" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A33" s="3"/>
-      <c r="B33" s="3"/>
-      <c r="C33" s="3"/>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-      <c r="G33" s="3"/>
-      <c r="H33" s="3"/>
-    </row>
-    <row r="34" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A34" s="3"/>
-      <c r="B34" s="3"/>
-      <c r="C34" s="3"/>
-      <c r="D34" s="3"/>
-      <c r="E34" s="3"/>
-      <c r="F34" s="3"/>
-      <c r="G34" s="3"/>
-      <c r="H34" s="3"/>
-    </row>
-    <row r="35" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A35" s="3"/>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
-      <c r="G35" s="3"/>
-      <c r="H35" s="3"/>
-    </row>
-    <row r="36" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A36" s="3"/>
-      <c r="B36" s="3"/>
-      <c r="C36" s="3"/>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
-      <c r="G36" s="3"/>
-      <c r="H36" s="3"/>
-    </row>
-    <row r="37" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A37" s="3"/>
-      <c r="B37" s="3"/>
-      <c r="C37" s="3"/>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-      <c r="G37" s="3"/>
-      <c r="H37" s="3"/>
-    </row>
-    <row r="38" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A38" s="3"/>
-      <c r="B38" s="3"/>
-      <c r="C38" s="3"/>
-      <c r="D38" s="3"/>
-      <c r="E38" s="3"/>
-      <c r="F38" s="3"/>
-      <c r="G38" s="3"/>
-      <c r="H38" s="3"/>
-    </row>
-    <row r="39" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A39" s="3"/>
-      <c r="B39" s="3"/>
-      <c r="C39" s="3"/>
-      <c r="D39" s="3"/>
-      <c r="E39" s="3"/>
-      <c r="F39" s="3"/>
-      <c r="G39" s="3"/>
-      <c r="H39" s="3"/>
+      <c r="H11" s="12" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A12" s="12"/>
+      <c r="B12" s="12"/>
+      <c r="C12" s="14"/>
+      <c r="D12" s="14"/>
+      <c r="E12" s="12"/>
+      <c r="F12" s="12"/>
+      <c r="G12" s="12"/>
+      <c r="H12" s="12"/>
+    </row>
+    <row r="13" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A13" s="12"/>
+      <c r="B13" s="12"/>
+      <c r="C13" s="12"/>
+      <c r="D13" s="12"/>
+      <c r="E13" s="12"/>
+      <c r="F13" s="12"/>
+      <c r="G13" s="12"/>
+      <c r="H13" s="12"/>
+    </row>
+    <row r="14" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A14" s="12"/>
+      <c r="B14" s="12"/>
+      <c r="C14" s="12"/>
+      <c r="D14" s="12"/>
+      <c r="E14" s="12"/>
+      <c r="F14" s="12"/>
+      <c r="G14" s="12"/>
+      <c r="H14" s="12"/>
+    </row>
+    <row r="15" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A15" s="12"/>
+      <c r="B15" s="12"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+    </row>
+    <row r="16" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A16" s="12"/>
+      <c r="B16" s="12"/>
+      <c r="C16" s="12"/>
+      <c r="D16" s="12"/>
+      <c r="E16" s="12"/>
+      <c r="F16" s="12"/>
+      <c r="G16" s="12"/>
+      <c r="H16" s="12"/>
+    </row>
+    <row r="17" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A17" s="12"/>
+      <c r="B17" s="12"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+    </row>
+    <row r="18" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A18" s="12"/>
+      <c r="B18" s="12"/>
+      <c r="C18" s="12"/>
+      <c r="D18" s="12"/>
+      <c r="E18" s="12"/>
+      <c r="F18" s="12"/>
+      <c r="G18" s="12"/>
+      <c r="H18" s="12"/>
+    </row>
+    <row r="19" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A19" s="12"/>
+      <c r="B19" s="12"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+    </row>
+    <row r="20" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A20" s="12"/>
+      <c r="B20" s="12"/>
+      <c r="C20" s="12"/>
+      <c r="D20" s="12"/>
+      <c r="E20" s="12"/>
+      <c r="F20" s="12"/>
+      <c r="G20" s="12"/>
+      <c r="H20" s="12"/>
+    </row>
+    <row r="21" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A21" s="12"/>
+      <c r="B21" s="12"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+    </row>
+    <row r="22" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A22" s="12"/>
+      <c r="B22" s="12"/>
+      <c r="C22" s="12"/>
+      <c r="D22" s="12"/>
+      <c r="E22" s="12"/>
+      <c r="F22" s="12"/>
+      <c r="G22" s="12"/>
+      <c r="H22" s="12"/>
+    </row>
+    <row r="23" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A23" s="12"/>
+      <c r="B23" s="12"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+    </row>
+    <row r="24" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A24" s="12"/>
+      <c r="B24" s="12"/>
+      <c r="C24" s="12"/>
+      <c r="D24" s="12"/>
+      <c r="E24" s="12"/>
+      <c r="F24" s="12"/>
+      <c r="G24" s="12"/>
+      <c r="H24" s="12"/>
+    </row>
+    <row r="25" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A25" s="12"/>
+      <c r="B25" s="12"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+    </row>
+    <row r="26" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A26" s="12"/>
+      <c r="B26" s="12"/>
+      <c r="C26" s="12"/>
+      <c r="D26" s="12"/>
+      <c r="E26" s="12"/>
+      <c r="F26" s="12"/>
+      <c r="G26" s="12"/>
+      <c r="H26" s="12"/>
+    </row>
+    <row r="27" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A27" s="12"/>
+      <c r="B27" s="12"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+    </row>
+    <row r="28" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A28" s="12"/>
+      <c r="B28" s="12"/>
+      <c r="C28" s="12"/>
+      <c r="D28" s="12"/>
+      <c r="E28" s="12"/>
+      <c r="F28" s="12"/>
+      <c r="G28" s="12"/>
+      <c r="H28" s="12"/>
+    </row>
+    <row r="29" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A29" s="12"/>
+      <c r="B29" s="12"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+    </row>
+    <row r="30" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A30" s="12"/>
+      <c r="B30" s="12"/>
+      <c r="C30" s="12"/>
+      <c r="D30" s="12"/>
+      <c r="E30" s="12"/>
+      <c r="F30" s="12"/>
+      <c r="G30" s="12"/>
+      <c r="H30" s="12"/>
+    </row>
+    <row r="31" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A31" s="12"/>
+      <c r="B31" s="12"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="12"/>
+    </row>
+    <row r="32" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A32" s="12"/>
+      <c r="B32" s="12"/>
+      <c r="C32" s="12"/>
+      <c r="D32" s="12"/>
+      <c r="E32" s="12"/>
+      <c r="F32" s="12"/>
+      <c r="G32" s="12"/>
+      <c r="H32" s="12"/>
+    </row>
+    <row r="33" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A33" s="12"/>
+      <c r="B33" s="12"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="12"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+    </row>
+    <row r="34" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A34" s="12"/>
+      <c r="B34" s="12"/>
+      <c r="C34" s="12"/>
+      <c r="D34" s="12"/>
+      <c r="E34" s="12"/>
+      <c r="F34" s="12"/>
+      <c r="G34" s="12"/>
+      <c r="H34" s="12"/>
+    </row>
+    <row r="35" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A35" s="12"/>
+      <c r="B35" s="12"/>
+      <c r="C35" s="12"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="12"/>
+      <c r="F35" s="12"/>
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+    </row>
+    <row r="36" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A36" s="12"/>
+      <c r="B36" s="12"/>
+      <c r="C36" s="12"/>
+      <c r="D36" s="12"/>
+      <c r="E36" s="12"/>
+      <c r="F36" s="12"/>
+      <c r="G36" s="12"/>
+      <c r="H36" s="12"/>
+    </row>
+    <row r="37" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A37" s="12"/>
+      <c r="B37" s="12"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+    </row>
+    <row r="38" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A38" s="12"/>
+      <c r="B38" s="12"/>
+      <c r="C38" s="12"/>
+      <c r="D38" s="12"/>
+      <c r="E38" s="12"/>
+      <c r="F38" s="12"/>
+      <c r="G38" s="12"/>
+      <c r="H38" s="12"/>
+    </row>
+    <row r="39" spans="1:8" ht="18" x14ac:dyDescent="0.3">
+      <c r="A39" s="12"/>
+      <c r="B39" s="12"/>
+      <c r="C39" s="12"/>
+      <c r="D39" s="12"/>
+      <c r="E39" s="12"/>
+      <c r="F39" s="12"/>
+      <c r="G39" s="12"/>
+      <c r="H39" s="12"/>
     </row>
     <row r="40" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A40" s="3"/>
@@ -2090,62 +2158,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="9"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="10"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="12" t="s">
+      <c r="B4" s="9"/>
+      <c r="C4" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10" t="s">
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
     </row>
     <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
@@ -2203,62 +2271,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="9"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="10"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="12" t="s">
+      <c r="B4" s="9"/>
+      <c r="C4" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10" t="s">
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
     </row>
     <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
@@ -2313,62 +2381,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
-      <c r="H1" s="10"/>
+      <c r="B1" s="9"/>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="9"/>
+      <c r="H1" s="9"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="9"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
-      <c r="H2" s="10"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="9"/>
+      <c r="E2" s="9"/>
+      <c r="F2" s="9"/>
+      <c r="G2" s="9"/>
+      <c r="H2" s="9"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="10"/>
-      <c r="B3" s="10"/>
-      <c r="C3" s="10"/>
-      <c r="D3" s="10"/>
-      <c r="E3" s="10"/>
-      <c r="F3" s="10"/>
-      <c r="G3" s="10"/>
-      <c r="H3" s="10"/>
+      <c r="A3" s="9"/>
+      <c r="B3" s="9"/>
+      <c r="C3" s="9"/>
+      <c r="D3" s="9"/>
+      <c r="E3" s="9"/>
+      <c r="F3" s="9"/>
+      <c r="G3" s="9"/>
+      <c r="H3" s="9"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="10" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="10"/>
-      <c r="C4" s="12" t="s">
+      <c r="B4" s="9"/>
+      <c r="C4" s="11" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="10"/>
-      <c r="E4" s="10"/>
-      <c r="F4" s="10" t="s">
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="10"/>
-      <c r="H4" s="10"/>
+      <c r="G4" s="9"/>
+      <c r="H4" s="9"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="10"/>
-      <c r="B5" s="10"/>
-      <c r="C5" s="10"/>
-      <c r="D5" s="10"/>
-      <c r="E5" s="10"/>
-      <c r="F5" s="10"/>
-      <c r="G5" s="10"/>
-      <c r="H5" s="10"/>
+      <c r="A5" s="9"/>
+      <c r="B5" s="9"/>
+      <c r="C5" s="9"/>
+      <c r="D5" s="9"/>
+      <c r="E5" s="9"/>
+      <c r="F5" s="9"/>
+      <c r="G5" s="9"/>
+      <c r="H5" s="9"/>
     </row>
     <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">

</xml_diff>

<commit_message>
Internal_Link_Testing and excel file
</commit_message>
<xml_diff>
--- a/wikipedia-Testing-ExcelSheet.xlsx
+++ b/wikipedia-Testing-ExcelSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECT\wikipedia_testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D038705E-A186-44E1-86AF-239036070716}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE8B51A2-384E-4271-BE3E-322FDBC0EA5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{23CE8EF5-60A8-44F8-8BB4-9FD29C3B8C6A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="42">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="48">
   <si>
     <t>Test Area / Functionality</t>
   </si>
@@ -267,6 +267,31 @@
 6. check table of content is visible or not
 7. click on Geography
 8. verify is it Geography or not</t>
+  </si>
+  <si>
+    <t>Internal_Link_Test.java</t>
+  </si>
+  <si>
+    <t>Internal Links</t>
+  </si>
+  <si>
+    <t>Check whether internal links work</t>
+  </si>
+  <si>
+    <t>Click an internal Wikipedia link</t>
+  </si>
+  <si>
+    <t>pass</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1. Open ChromeBrowser
+2. Go to Wikipedia
+3. Search India
+4. click search button
+5. click on any internal link (link south asia)
+6. check result 
+7. quit
+</t>
   </si>
 </sst>
 </file>
@@ -348,13 +373,22 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -380,18 +414,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -721,71 +743,71 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="7" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="5"/>
-      <c r="E1" s="5"/>
-      <c r="F1" s="5"/>
-      <c r="G1" s="5"/>
-      <c r="H1" s="5"/>
+      <c r="B1" s="8"/>
+      <c r="C1" s="8"/>
+      <c r="D1" s="8"/>
+      <c r="E1" s="8"/>
+      <c r="F1" s="8"/>
+      <c r="G1" s="8"/>
+      <c r="H1" s="8"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="4"/>
-      <c r="B2" s="5"/>
-      <c r="C2" s="5"/>
-      <c r="D2" s="5"/>
-      <c r="E2" s="5"/>
-      <c r="F2" s="5"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
+      <c r="A2" s="7"/>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
+      <c r="H2" s="8"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="5"/>
-      <c r="B3" s="5"/>
-      <c r="C3" s="5"/>
-      <c r="D3" s="5"/>
-      <c r="E3" s="5"/>
-      <c r="F3" s="5"/>
-      <c r="G3" s="5"/>
-      <c r="H3" s="5"/>
+      <c r="A3" s="8"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
+      <c r="H3" s="8"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="6" t="s">
+      <c r="A4" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="5"/>
-      <c r="C4" s="7" t="s">
+      <c r="B4" s="8"/>
+      <c r="C4" s="10" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
-      <c r="F4" s="5" t="s">
+      <c r="D4" s="8"/>
+      <c r="E4" s="8"/>
+      <c r="F4" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
+      <c r="G4" s="8"/>
+      <c r="H4" s="8"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="5"/>
-      <c r="B5" s="5"/>
-      <c r="C5" s="5"/>
-      <c r="D5" s="5"/>
-      <c r="E5" s="5"/>
-      <c r="F5" s="5"/>
-      <c r="G5" s="5"/>
-      <c r="H5" s="5"/>
+      <c r="A5" s="8"/>
+      <c r="B5" s="8"/>
+      <c r="C5" s="8"/>
+      <c r="D5" s="8"/>
+      <c r="E5" s="8"/>
+      <c r="F5" s="8"/>
+      <c r="G5" s="8"/>
+      <c r="H5" s="8"/>
     </row>
     <row r="6" spans="1:8" ht="40.799999999999997" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="C6" s="15" t="s">
+      <c r="C6" s="6" t="s">
         <v>0</v>
       </c>
       <c r="D6" s="2" t="s">
@@ -805,410 +827,430 @@
       </c>
     </row>
     <row r="7" spans="1:8" ht="108" x14ac:dyDescent="0.3">
-      <c r="A7" s="12">
+      <c r="A7" s="4">
         <v>1</v>
       </c>
-      <c r="B7" s="12" t="s">
+      <c r="B7" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C7" s="12" t="s">
+      <c r="C7" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D7" s="12" t="s">
+      <c r="D7" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="E7" s="12" t="s">
+      <c r="E7" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="F7" s="13" t="s">
+      <c r="F7" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="G7" s="12" t="s">
+      <c r="G7" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H7" s="12" t="s">
+      <c r="H7" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="162" x14ac:dyDescent="0.3">
-      <c r="A8" s="12">
+      <c r="A8" s="4">
         <v>2</v>
       </c>
-      <c r="B8" s="12" t="s">
+      <c r="B8" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C8" s="12" t="s">
+      <c r="C8" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D8" s="12" t="s">
+      <c r="D8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="E8" s="12" t="s">
+      <c r="E8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="F8" s="13" t="s">
+      <c r="F8" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="G8" s="12" t="s">
+      <c r="G8" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H8" s="12" t="s">
+      <c r="H8" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="108" x14ac:dyDescent="0.3">
-      <c r="A9" s="12">
+      <c r="A9" s="4">
         <v>3</v>
       </c>
-      <c r="B9" s="12" t="s">
+      <c r="B9" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C9" s="12" t="s">
+      <c r="C9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D9" s="12" t="s">
+      <c r="D9" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E9" s="12" t="s">
+      <c r="E9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F9" s="13" t="s">
+      <c r="F9" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="G9" s="12" t="s">
+      <c r="G9" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H9" s="12" t="s">
+      <c r="H9" s="4" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="132" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="12"/>
-      <c r="B10" s="12" t="s">
+      <c r="A10" s="4">
+        <v>4</v>
+      </c>
+      <c r="B10" s="4" t="s">
         <v>31</v>
       </c>
-      <c r="C10" s="12" t="s">
+      <c r="C10" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D10" s="12" t="s">
+      <c r="D10" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="E10" s="12" t="s">
+      <c r="E10" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="F10" s="13" t="s">
+      <c r="F10" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="G10" s="12" t="s">
+      <c r="G10" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H10" s="12" t="s">
+      <c r="H10" s="4" t="s">
         <v>38</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="162" x14ac:dyDescent="0.3">
-      <c r="A11" s="12"/>
-      <c r="B11" s="12" t="s">
+      <c r="A11" s="4">
+        <v>5</v>
+      </c>
+      <c r="B11" s="4" t="s">
         <v>35</v>
       </c>
-      <c r="C11" s="12" t="s">
+      <c r="C11" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="D11" s="12" t="s">
+      <c r="D11" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="E11" s="12" t="s">
+      <c r="E11" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="F11" s="13" t="s">
+      <c r="F11" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="G11" s="12" t="s">
+      <c r="G11" s="4" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="12" t="s">
+      <c r="H11" s="4" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="12" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A12" s="12"/>
-      <c r="B12" s="12"/>
-      <c r="C12" s="14"/>
-      <c r="D12" s="14"/>
-      <c r="E12" s="12"/>
-      <c r="F12" s="12"/>
-      <c r="G12" s="12"/>
-      <c r="H12" s="12"/>
+    <row r="12" spans="1:8" ht="162" x14ac:dyDescent="0.3">
+      <c r="A12" s="4">
+        <v>6</v>
+      </c>
+      <c r="B12" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="E12" s="4" t="s">
+        <v>45</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="G12" s="4" t="s">
+        <v>46</v>
+      </c>
+      <c r="H12" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="13" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A13" s="12"/>
-      <c r="B13" s="12"/>
-      <c r="C13" s="12"/>
-      <c r="D13" s="12"/>
-      <c r="E13" s="12"/>
-      <c r="F13" s="12"/>
-      <c r="G13" s="12"/>
-      <c r="H13" s="12"/>
+      <c r="A13" s="4"/>
+      <c r="B13" s="4"/>
+      <c r="C13" s="4"/>
+      <c r="D13" s="4"/>
+      <c r="E13" s="4"/>
+      <c r="F13" s="4"/>
+      <c r="G13" s="4"/>
+      <c r="H13" s="4"/>
     </row>
     <row r="14" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A14" s="12"/>
-      <c r="B14" s="12"/>
-      <c r="C14" s="12"/>
-      <c r="D14" s="12"/>
-      <c r="E14" s="12"/>
-      <c r="F14" s="12"/>
-      <c r="G14" s="12"/>
-      <c r="H14" s="12"/>
+      <c r="A14" s="4"/>
+      <c r="B14" s="4"/>
+      <c r="C14" s="4"/>
+      <c r="D14" s="4"/>
+      <c r="E14" s="4"/>
+      <c r="F14" s="4"/>
+      <c r="G14" s="4"/>
+      <c r="H14" s="4"/>
     </row>
     <row r="15" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A15" s="12"/>
-      <c r="B15" s="12"/>
-      <c r="C15" s="12"/>
-      <c r="D15" s="12"/>
-      <c r="E15" s="12"/>
-      <c r="F15" s="12"/>
-      <c r="G15" s="12"/>
-      <c r="H15" s="12"/>
+      <c r="A15" s="4"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
+      <c r="F15" s="4"/>
+      <c r="G15" s="4"/>
+      <c r="H15" s="4"/>
     </row>
     <row r="16" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A16" s="12"/>
-      <c r="B16" s="12"/>
-      <c r="C16" s="12"/>
-      <c r="D16" s="12"/>
-      <c r="E16" s="12"/>
-      <c r="F16" s="12"/>
-      <c r="G16" s="12"/>
-      <c r="H16" s="12"/>
+      <c r="A16" s="4"/>
+      <c r="B16" s="4"/>
+      <c r="C16" s="4"/>
+      <c r="D16" s="4"/>
+      <c r="E16" s="4"/>
+      <c r="F16" s="4"/>
+      <c r="G16" s="4"/>
+      <c r="H16" s="4"/>
     </row>
     <row r="17" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A17" s="12"/>
-      <c r="B17" s="12"/>
-      <c r="C17" s="12"/>
-      <c r="D17" s="12"/>
-      <c r="E17" s="12"/>
-      <c r="F17" s="12"/>
-      <c r="G17" s="12"/>
-      <c r="H17" s="12"/>
+      <c r="A17" s="4"/>
+      <c r="B17" s="4"/>
+      <c r="C17" s="4"/>
+      <c r="D17" s="4"/>
+      <c r="E17" s="4"/>
+      <c r="F17" s="4"/>
+      <c r="G17" s="4"/>
+      <c r="H17" s="4"/>
     </row>
     <row r="18" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A18" s="12"/>
-      <c r="B18" s="12"/>
-      <c r="C18" s="12"/>
-      <c r="D18" s="12"/>
-      <c r="E18" s="12"/>
-      <c r="F18" s="12"/>
-      <c r="G18" s="12"/>
-      <c r="H18" s="12"/>
+      <c r="A18" s="4"/>
+      <c r="B18" s="4"/>
+      <c r="C18" s="4"/>
+      <c r="D18" s="4"/>
+      <c r="E18" s="4"/>
+      <c r="F18" s="4"/>
+      <c r="G18" s="4"/>
+      <c r="H18" s="4"/>
     </row>
     <row r="19" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A19" s="12"/>
-      <c r="B19" s="12"/>
-      <c r="C19" s="12"/>
-      <c r="D19" s="12"/>
-      <c r="E19" s="12"/>
-      <c r="F19" s="12"/>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
+      <c r="A19" s="4"/>
+      <c r="B19" s="4"/>
+      <c r="C19" s="4"/>
+      <c r="D19" s="4"/>
+      <c r="E19" s="4"/>
+      <c r="F19" s="4"/>
+      <c r="G19" s="4"/>
+      <c r="H19" s="4"/>
     </row>
     <row r="20" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A20" s="12"/>
-      <c r="B20" s="12"/>
-      <c r="C20" s="12"/>
-      <c r="D20" s="12"/>
-      <c r="E20" s="12"/>
-      <c r="F20" s="12"/>
-      <c r="G20" s="12"/>
-      <c r="H20" s="12"/>
+      <c r="A20" s="4"/>
+      <c r="B20" s="4"/>
+      <c r="C20" s="4"/>
+      <c r="D20" s="4"/>
+      <c r="E20" s="4"/>
+      <c r="F20" s="4"/>
+      <c r="G20" s="4"/>
+      <c r="H20" s="4"/>
     </row>
     <row r="21" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A21" s="12"/>
-      <c r="B21" s="12"/>
-      <c r="C21" s="12"/>
-      <c r="D21" s="12"/>
-      <c r="E21" s="12"/>
-      <c r="F21" s="12"/>
-      <c r="G21" s="12"/>
-      <c r="H21" s="12"/>
+      <c r="A21" s="4"/>
+      <c r="B21" s="4"/>
+      <c r="C21" s="4"/>
+      <c r="D21" s="4"/>
+      <c r="E21" s="4"/>
+      <c r="F21" s="4"/>
+      <c r="G21" s="4"/>
+      <c r="H21" s="4"/>
     </row>
     <row r="22" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A22" s="12"/>
-      <c r="B22" s="12"/>
-      <c r="C22" s="12"/>
-      <c r="D22" s="12"/>
-      <c r="E22" s="12"/>
-      <c r="F22" s="12"/>
-      <c r="G22" s="12"/>
-      <c r="H22" s="12"/>
+      <c r="A22" s="4"/>
+      <c r="B22" s="4"/>
+      <c r="C22" s="4"/>
+      <c r="D22" s="4"/>
+      <c r="E22" s="4"/>
+      <c r="F22" s="4"/>
+      <c r="G22" s="4"/>
+      <c r="H22" s="4"/>
     </row>
     <row r="23" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A23" s="12"/>
-      <c r="B23" s="12"/>
-      <c r="C23" s="12"/>
-      <c r="D23" s="12"/>
-      <c r="E23" s="12"/>
-      <c r="F23" s="12"/>
-      <c r="G23" s="12"/>
-      <c r="H23" s="12"/>
+      <c r="A23" s="4"/>
+      <c r="B23" s="4"/>
+      <c r="C23" s="4"/>
+      <c r="D23" s="4"/>
+      <c r="E23" s="4"/>
+      <c r="F23" s="4"/>
+      <c r="G23" s="4"/>
+      <c r="H23" s="4"/>
     </row>
     <row r="24" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A24" s="12"/>
-      <c r="B24" s="12"/>
-      <c r="C24" s="12"/>
-      <c r="D24" s="12"/>
-      <c r="E24" s="12"/>
-      <c r="F24" s="12"/>
-      <c r="G24" s="12"/>
-      <c r="H24" s="12"/>
+      <c r="A24" s="4"/>
+      <c r="B24" s="4"/>
+      <c r="C24" s="4"/>
+      <c r="D24" s="4"/>
+      <c r="E24" s="4"/>
+      <c r="F24" s="4"/>
+      <c r="G24" s="4"/>
+      <c r="H24" s="4"/>
     </row>
     <row r="25" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A25" s="12"/>
-      <c r="B25" s="12"/>
-      <c r="C25" s="12"/>
-      <c r="D25" s="12"/>
-      <c r="E25" s="12"/>
-      <c r="F25" s="12"/>
-      <c r="G25" s="12"/>
-      <c r="H25" s="12"/>
+      <c r="A25" s="4"/>
+      <c r="B25" s="4"/>
+      <c r="C25" s="4"/>
+      <c r="D25" s="4"/>
+      <c r="E25" s="4"/>
+      <c r="F25" s="4"/>
+      <c r="G25" s="4"/>
+      <c r="H25" s="4"/>
     </row>
     <row r="26" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A26" s="12"/>
-      <c r="B26" s="12"/>
-      <c r="C26" s="12"/>
-      <c r="D26" s="12"/>
-      <c r="E26" s="12"/>
-      <c r="F26" s="12"/>
-      <c r="G26" s="12"/>
-      <c r="H26" s="12"/>
+      <c r="A26" s="4"/>
+      <c r="B26" s="4"/>
+      <c r="C26" s="4"/>
+      <c r="D26" s="4"/>
+      <c r="E26" s="4"/>
+      <c r="F26" s="4"/>
+      <c r="G26" s="4"/>
+      <c r="H26" s="4"/>
     </row>
     <row r="27" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A27" s="12"/>
-      <c r="B27" s="12"/>
-      <c r="C27" s="12"/>
-      <c r="D27" s="12"/>
-      <c r="E27" s="12"/>
-      <c r="F27" s="12"/>
-      <c r="G27" s="12"/>
-      <c r="H27" s="12"/>
+      <c r="A27" s="4"/>
+      <c r="B27" s="4"/>
+      <c r="C27" s="4"/>
+      <c r="D27" s="4"/>
+      <c r="E27" s="4"/>
+      <c r="F27" s="4"/>
+      <c r="G27" s="4"/>
+      <c r="H27" s="4"/>
     </row>
     <row r="28" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A28" s="12"/>
-      <c r="B28" s="12"/>
-      <c r="C28" s="12"/>
-      <c r="D28" s="12"/>
-      <c r="E28" s="12"/>
-      <c r="F28" s="12"/>
-      <c r="G28" s="12"/>
-      <c r="H28" s="12"/>
+      <c r="A28" s="4"/>
+      <c r="B28" s="4"/>
+      <c r="C28" s="4"/>
+      <c r="D28" s="4"/>
+      <c r="E28" s="4"/>
+      <c r="F28" s="4"/>
+      <c r="G28" s="4"/>
+      <c r="H28" s="4"/>
     </row>
     <row r="29" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A29" s="12"/>
-      <c r="B29" s="12"/>
-      <c r="C29" s="12"/>
-      <c r="D29" s="12"/>
-      <c r="E29" s="12"/>
-      <c r="F29" s="12"/>
-      <c r="G29" s="12"/>
-      <c r="H29" s="12"/>
+      <c r="A29" s="4"/>
+      <c r="B29" s="4"/>
+      <c r="C29" s="4"/>
+      <c r="D29" s="4"/>
+      <c r="E29" s="4"/>
+      <c r="F29" s="4"/>
+      <c r="G29" s="4"/>
+      <c r="H29" s="4"/>
     </row>
     <row r="30" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A30" s="12"/>
-      <c r="B30" s="12"/>
-      <c r="C30" s="12"/>
-      <c r="D30" s="12"/>
-      <c r="E30" s="12"/>
-      <c r="F30" s="12"/>
-      <c r="G30" s="12"/>
-      <c r="H30" s="12"/>
+      <c r="A30" s="4"/>
+      <c r="B30" s="4"/>
+      <c r="C30" s="4"/>
+      <c r="D30" s="4"/>
+      <c r="E30" s="4"/>
+      <c r="F30" s="4"/>
+      <c r="G30" s="4"/>
+      <c r="H30" s="4"/>
     </row>
     <row r="31" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A31" s="12"/>
-      <c r="B31" s="12"/>
-      <c r="C31" s="12"/>
-      <c r="D31" s="12"/>
-      <c r="E31" s="12"/>
-      <c r="F31" s="12"/>
-      <c r="G31" s="12"/>
-      <c r="H31" s="12"/>
+      <c r="A31" s="4"/>
+      <c r="B31" s="4"/>
+      <c r="C31" s="4"/>
+      <c r="D31" s="4"/>
+      <c r="E31" s="4"/>
+      <c r="F31" s="4"/>
+      <c r="G31" s="4"/>
+      <c r="H31" s="4"/>
     </row>
     <row r="32" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A32" s="12"/>
-      <c r="B32" s="12"/>
-      <c r="C32" s="12"/>
-      <c r="D32" s="12"/>
-      <c r="E32" s="12"/>
-      <c r="F32" s="12"/>
-      <c r="G32" s="12"/>
-      <c r="H32" s="12"/>
+      <c r="A32" s="4"/>
+      <c r="B32" s="4"/>
+      <c r="C32" s="4"/>
+      <c r="D32" s="4"/>
+      <c r="E32" s="4"/>
+      <c r="F32" s="4"/>
+      <c r="G32" s="4"/>
+      <c r="H32" s="4"/>
     </row>
     <row r="33" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A33" s="12"/>
-      <c r="B33" s="12"/>
-      <c r="C33" s="12"/>
-      <c r="D33" s="12"/>
-      <c r="E33" s="12"/>
-      <c r="F33" s="12"/>
-      <c r="G33" s="12"/>
-      <c r="H33" s="12"/>
+      <c r="A33" s="4"/>
+      <c r="B33" s="4"/>
+      <c r="C33" s="4"/>
+      <c r="D33" s="4"/>
+      <c r="E33" s="4"/>
+      <c r="F33" s="4"/>
+      <c r="G33" s="4"/>
+      <c r="H33" s="4"/>
     </row>
     <row r="34" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A34" s="12"/>
-      <c r="B34" s="12"/>
-      <c r="C34" s="12"/>
-      <c r="D34" s="12"/>
-      <c r="E34" s="12"/>
-      <c r="F34" s="12"/>
-      <c r="G34" s="12"/>
-      <c r="H34" s="12"/>
+      <c r="A34" s="4"/>
+      <c r="B34" s="4"/>
+      <c r="C34" s="4"/>
+      <c r="D34" s="4"/>
+      <c r="E34" s="4"/>
+      <c r="F34" s="4"/>
+      <c r="G34" s="4"/>
+      <c r="H34" s="4"/>
     </row>
     <row r="35" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A35" s="12"/>
-      <c r="B35" s="12"/>
-      <c r="C35" s="12"/>
-      <c r="D35" s="12"/>
-      <c r="E35" s="12"/>
-      <c r="F35" s="12"/>
-      <c r="G35" s="12"/>
-      <c r="H35" s="12"/>
+      <c r="A35" s="4"/>
+      <c r="B35" s="4"/>
+      <c r="C35" s="4"/>
+      <c r="D35" s="4"/>
+      <c r="E35" s="4"/>
+      <c r="F35" s="4"/>
+      <c r="G35" s="4"/>
+      <c r="H35" s="4"/>
     </row>
     <row r="36" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A36" s="12"/>
-      <c r="B36" s="12"/>
-      <c r="C36" s="12"/>
-      <c r="D36" s="12"/>
-      <c r="E36" s="12"/>
-      <c r="F36" s="12"/>
-      <c r="G36" s="12"/>
-      <c r="H36" s="12"/>
+      <c r="A36" s="4"/>
+      <c r="B36" s="4"/>
+      <c r="C36" s="4"/>
+      <c r="D36" s="4"/>
+      <c r="E36" s="4"/>
+      <c r="F36" s="4"/>
+      <c r="G36" s="4"/>
+      <c r="H36" s="4"/>
     </row>
     <row r="37" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A37" s="12"/>
-      <c r="B37" s="12"/>
-      <c r="C37" s="12"/>
-      <c r="D37" s="12"/>
-      <c r="E37" s="12"/>
-      <c r="F37" s="12"/>
-      <c r="G37" s="12"/>
-      <c r="H37" s="12"/>
+      <c r="A37" s="4"/>
+      <c r="B37" s="4"/>
+      <c r="C37" s="4"/>
+      <c r="D37" s="4"/>
+      <c r="E37" s="4"/>
+      <c r="F37" s="4"/>
+      <c r="G37" s="4"/>
+      <c r="H37" s="4"/>
     </row>
     <row r="38" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A38" s="12"/>
-      <c r="B38" s="12"/>
-      <c r="C38" s="12"/>
-      <c r="D38" s="12"/>
-      <c r="E38" s="12"/>
-      <c r="F38" s="12"/>
-      <c r="G38" s="12"/>
-      <c r="H38" s="12"/>
+      <c r="A38" s="4"/>
+      <c r="B38" s="4"/>
+      <c r="C38" s="4"/>
+      <c r="D38" s="4"/>
+      <c r="E38" s="4"/>
+      <c r="F38" s="4"/>
+      <c r="G38" s="4"/>
+      <c r="H38" s="4"/>
     </row>
     <row r="39" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A39" s="12"/>
-      <c r="B39" s="12"/>
-      <c r="C39" s="12"/>
-      <c r="D39" s="12"/>
-      <c r="E39" s="12"/>
-      <c r="F39" s="12"/>
-      <c r="G39" s="12"/>
-      <c r="H39" s="12"/>
+      <c r="A39" s="4"/>
+      <c r="B39" s="4"/>
+      <c r="C39" s="4"/>
+      <c r="D39" s="4"/>
+      <c r="E39" s="4"/>
+      <c r="F39" s="4"/>
+      <c r="G39" s="4"/>
+      <c r="H39" s="4"/>
     </row>
     <row r="40" spans="1:8" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A40" s="3"/>
@@ -2158,62 +2200,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="8"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="11" t="s">
+      <c r="B4" s="12"/>
+      <c r="C4" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9" t="s">
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12" t="s">
         <v>12</v>
       </c>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
+      <c r="A5" s="12"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
     </row>
     <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
@@ -2271,62 +2313,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="8"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="11" t="s">
+      <c r="B4" s="12"/>
+      <c r="C4" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9" t="s">
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
+      <c r="A5" s="12"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
     </row>
     <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
@@ -2381,62 +2423,62 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="8" t="s">
+      <c r="A1" s="11" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="9"/>
-      <c r="C1" s="9"/>
-      <c r="D1" s="9"/>
-      <c r="E1" s="9"/>
-      <c r="F1" s="9"/>
-      <c r="G1" s="9"/>
-      <c r="H1" s="9"/>
+      <c r="B1" s="12"/>
+      <c r="C1" s="12"/>
+      <c r="D1" s="12"/>
+      <c r="E1" s="12"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="12"/>
+      <c r="H1" s="12"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="8"/>
-      <c r="B2" s="9"/>
-      <c r="C2" s="9"/>
-      <c r="D2" s="9"/>
-      <c r="E2" s="9"/>
-      <c r="F2" s="9"/>
-      <c r="G2" s="9"/>
-      <c r="H2" s="9"/>
+      <c r="A2" s="11"/>
+      <c r="B2" s="12"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="12"/>
+      <c r="H2" s="12"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="9"/>
-      <c r="B3" s="9"/>
-      <c r="C3" s="9"/>
-      <c r="D3" s="9"/>
-      <c r="E3" s="9"/>
-      <c r="F3" s="9"/>
-      <c r="G3" s="9"/>
-      <c r="H3" s="9"/>
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="12"/>
+      <c r="D3" s="12"/>
+      <c r="E3" s="12"/>
+      <c r="F3" s="12"/>
+      <c r="G3" s="12"/>
+      <c r="H3" s="12"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="10" t="s">
+      <c r="A4" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="B4" s="9"/>
-      <c r="C4" s="11" t="s">
+      <c r="B4" s="12"/>
+      <c r="C4" s="14" t="s">
         <v>11</v>
       </c>
-      <c r="D4" s="9"/>
-      <c r="E4" s="9"/>
-      <c r="F4" s="9" t="s">
+      <c r="D4" s="12"/>
+      <c r="E4" s="12"/>
+      <c r="F4" s="12" t="s">
         <v>10</v>
       </c>
-      <c r="G4" s="9"/>
-      <c r="H4" s="9"/>
+      <c r="G4" s="12"/>
+      <c r="H4" s="12"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="9"/>
-      <c r="B5" s="9"/>
-      <c r="C5" s="9"/>
-      <c r="D5" s="9"/>
-      <c r="E5" s="9"/>
-      <c r="F5" s="9"/>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9"/>
+      <c r="A5" s="12"/>
+      <c r="B5" s="12"/>
+      <c r="C5" s="12"/>
+      <c r="D5" s="12"/>
+      <c r="E5" s="12"/>
+      <c r="F5" s="12"/>
+      <c r="G5" s="12"/>
+      <c r="H5" s="12"/>
     </row>
     <row r="6" spans="1:8" ht="18" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">

</xml_diff>

<commit_message>
adding External Links Testing and excel file
</commit_message>
<xml_diff>
--- a/wikipedia-Testing-ExcelSheet.xlsx
+++ b/wikipedia-Testing-ExcelSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECT\wikipedia_testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE8B51A2-384E-4271-BE3E-322FDBC0EA5E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DD9CF82-582A-46C3-B3AA-1C1DBE92FF0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{23CE8EF5-60A8-44F8-8BB4-9FD29C3B8C6A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="52">
   <si>
     <t>Test Area / Functionality</t>
   </si>
@@ -281,9 +281,6 @@
     <t>Click an internal Wikipedia link</t>
   </si>
   <si>
-    <t>pass</t>
-  </si>
-  <si>
     <t xml:space="preserve">1. Open ChromeBrowser
 2. Go to Wikipedia
 3. Search India
@@ -292,6 +289,26 @@
 6. check result 
 7. quit
 </t>
+  </si>
+  <si>
+    <t xml:space="preserve"> External_Links_Test.java</t>
+  </si>
+  <si>
+    <t>External Links</t>
+  </si>
+  <si>
+    <t>Check whether external links work</t>
+  </si>
+  <si>
+    <t>Click an external link</t>
+  </si>
+  <si>
+    <t>1. Open ChromeBrowser
+2. Go to Wikipedia
+3. Search india
+4. click search button
+5. click on External link
+6. check the status is it open or not</t>
   </si>
 </sst>
 </file>
@@ -973,24 +990,40 @@
         <v>45</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G12" s="4" t="s">
-        <v>46</v>
+        <v>21</v>
       </c>
       <c r="H12" s="4" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="13" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A13" s="4"/>
-      <c r="B13" s="4"/>
-      <c r="C13" s="4"/>
-      <c r="D13" s="4"/>
-      <c r="E13" s="4"/>
-      <c r="F13" s="4"/>
-      <c r="G13" s="4"/>
-      <c r="H13" s="4"/>
+    <row r="13" spans="1:8" ht="126" x14ac:dyDescent="0.3">
+      <c r="A13" s="4">
+        <v>7</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>47</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>49</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="G13" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H13" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="14" spans="1:8" ht="18" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>

</xml_diff>

<commit_message>
adding references testing and their excel file
</commit_message>
<xml_diff>
--- a/wikipedia-Testing-ExcelSheet.xlsx
+++ b/wikipedia-Testing-ExcelSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECT\wikipedia_testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6DD9CF82-582A-46C3-B3AA-1C1DBE92FF0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{60B11E3E-1AAF-478F-98B7-B5ED0A9F29E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{23CE8EF5-60A8-44F8-8BB4-9FD29C3B8C6A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="57">
   <si>
     <t>Test Area / Functionality</t>
   </si>
@@ -309,6 +309,27 @@
 4. click search button
 5. click on External link
 6. check the status is it open or not</t>
+  </si>
+  <si>
+    <t>References_test.java</t>
+  </si>
+  <si>
+    <t>References</t>
+  </si>
+  <si>
+    <t>Check whether references are displayed</t>
+  </si>
+  <si>
+    <t>Open a reference from the article</t>
+  </si>
+  <si>
+    <t>1.Open ChromeBrowser
+2.Go to Wikipedia
+3. Seaarch India
+4. Click search button
+5. click on references
+6. click on any Reference link
+7. Verify the reference content is displayed or not</t>
   </si>
 </sst>
 </file>
@@ -1025,15 +1046,31 @@
         <v>20</v>
       </c>
     </row>
-    <row r="14" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A14" s="4"/>
-      <c r="B14" s="4"/>
-      <c r="C14" s="4"/>
-      <c r="D14" s="4"/>
-      <c r="E14" s="4"/>
-      <c r="F14" s="4"/>
-      <c r="G14" s="4"/>
-      <c r="H14" s="4"/>
+    <row r="14" spans="1:8" ht="144" x14ac:dyDescent="0.3">
+      <c r="A14" s="4">
+        <v>8</v>
+      </c>
+      <c r="B14" s="4" t="s">
+        <v>52</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D14" s="4" t="s">
+        <v>54</v>
+      </c>
+      <c r="E14" s="4" t="s">
+        <v>55</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="G14" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="H14" s="4" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="15" spans="1:8" ht="18" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>

</xml_diff>

<commit_message>
adding images Testing and there Excel row
</commit_message>
<xml_diff>
--- a/wikipedia-Testing-ExcelSheet.xlsx
+++ b/wikipedia-Testing-ExcelSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECT\wikipedia_testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE7F1590-1827-4C55-8099-D6B79CA593A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D31E658-FF41-4B59-87F8-C944D0BA5008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{23CE8EF5-60A8-44F8-8BB4-9FD29C3B8C6A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="57">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="62">
   <si>
     <t>Test Area / Functionality</t>
   </si>
@@ -330,6 +330,27 @@
   </si>
   <si>
     <t>Test status (Pass/Fail)</t>
+  </si>
+  <si>
+    <t>Images_Test.java</t>
+  </si>
+  <si>
+    <t>Images</t>
+  </si>
+  <si>
+    <t>Check whether article images are displayed</t>
+  </si>
+  <si>
+    <t>Open an article and check images</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.Open ChromeBrowser
+2.Go to Wikipedia
+3. Seaarch India
+4. Click search button
+5. click on Image
+6. check it is display or not.
+7. Verify </t>
   </si>
 </sst>
 </file>
@@ -1072,15 +1093,31 @@
         <v>19</v>
       </c>
     </row>
-    <row r="15" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A15" s="4"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-      <c r="F15" s="4"/>
-      <c r="G15" s="4"/>
-      <c r="H15" s="4"/>
+    <row r="15" spans="1:8" ht="126" x14ac:dyDescent="0.3">
+      <c r="A15" s="4">
+        <v>9</v>
+      </c>
+      <c r="B15" s="4" t="s">
+        <v>57</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>58</v>
+      </c>
+      <c r="D15" s="4" t="s">
+        <v>59</v>
+      </c>
+      <c r="E15" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="F15" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="G15" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H15" s="4" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="16" spans="1:8" ht="18" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>

</xml_diff>

<commit_message>
adding HomeNavigation Test and there Excel File
</commit_message>
<xml_diff>
--- a/wikipedia-Testing-ExcelSheet.xlsx
+++ b/wikipedia-Testing-ExcelSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECT\wikipedia_testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D31E658-FF41-4B59-87F8-C944D0BA5008}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57826F2C-E5EA-460D-8709-92BE61D4089C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{23CE8EF5-60A8-44F8-8BB4-9FD29C3B8C6A}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="67">
   <si>
     <t>Test Area / Functionality</t>
   </si>
@@ -351,6 +351,26 @@
 5. click on Image
 6. check it is display or not.
 7. Verify </t>
+  </si>
+  <si>
+    <t>HomeNavigationTest.java</t>
+  </si>
+  <si>
+    <t>Home Page Navigation</t>
+  </si>
+  <si>
+    <t>Check whether Wikipedia home page opens</t>
+  </si>
+  <si>
+    <t>Open Wikipedia home page</t>
+  </si>
+  <si>
+    <t>1.Open ChromeBrowser
+2.Go to Wikipedia
+3. Check Homepage is visible or not
+4. Check Searchbar is visible or not
+5. Check SearchButton is visible or not
+6. Quit.</t>
   </si>
 </sst>
 </file>
@@ -796,7 +816,7 @@
     <col min="3" max="3" width="20.44140625" customWidth="1"/>
     <col min="4" max="4" width="23.88671875" customWidth="1"/>
     <col min="5" max="5" width="24.44140625" customWidth="1"/>
-    <col min="6" max="6" width="33.6640625" customWidth="1"/>
+    <col min="6" max="6" width="40.44140625" customWidth="1"/>
     <col min="7" max="7" width="20.6640625" customWidth="1"/>
     <col min="8" max="8" width="31.5546875" customWidth="1"/>
   </cols>
@@ -1119,15 +1139,31 @@
         <v>19</v>
       </c>
     </row>
-    <row r="16" spans="1:8" ht="18" x14ac:dyDescent="0.3">
-      <c r="A16" s="4"/>
-      <c r="B16" s="4"/>
-      <c r="C16" s="4"/>
-      <c r="D16" s="4"/>
-      <c r="E16" s="4"/>
-      <c r="F16" s="4"/>
-      <c r="G16" s="4"/>
-      <c r="H16" s="4"/>
+    <row r="16" spans="1:8" ht="126" x14ac:dyDescent="0.3">
+      <c r="A16" s="4">
+        <v>10</v>
+      </c>
+      <c r="B16" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D16" s="4" t="s">
+        <v>64</v>
+      </c>
+      <c r="E16" s="4" t="s">
+        <v>65</v>
+      </c>
+      <c r="F16" s="5" t="s">
+        <v>66</v>
+      </c>
+      <c r="G16" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="H16" s="4" t="s">
+        <v>19</v>
+      </c>
     </row>
     <row r="17" spans="1:8" ht="18" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>

</xml_diff>

<commit_message>
Add refresh Button Testing of the article page in file Refresh_Button_Test.java , Test is pass && Add Test step ,Test Scenario and status of test in wikipedia-Testing-ExcelSheet.xlsx file
</commit_message>
<xml_diff>
--- a/wikipedia-Testing-ExcelSheet.xlsx
+++ b/wikipedia-Testing-ExcelSheet.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="30430"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECT\wikipedia_testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6AB75A56-3E5D-43AE-929D-415D2FFCF5DE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B524CD51-B1C7-45C7-AF58-783C80DC38E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="82">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="79">
   <si>
     <t>Wikipedia Search &amp; Reader UI</t>
   </si>
@@ -115,9 +115,6 @@
     <t>Article_Page_Test.java</t>
   </si>
   <si>
-    <t>Article Title</t>
-  </si>
-  <si>
     <t>Check article title after opening an article</t>
   </si>
   <si>
@@ -174,9 +171,6 @@
   </si>
   <si>
     <t>Table_of_Content_test.java</t>
-  </si>
-  <si>
-    <t>Table of Contents</t>
   </si>
   <si>
     <t>Check whether Table of Contents is displayed</t>
@@ -218,9 +212,6 @@
     <t>Internal_Link_Test.java</t>
   </si>
   <si>
-    <t>Internal Links</t>
-  </si>
-  <si>
     <t>Check whether internal links work</t>
   </si>
   <si>
@@ -240,9 +231,6 @@
     <t xml:space="preserve"> External_Links_Test.java</t>
   </si>
   <si>
-    <t>External Links</t>
-  </si>
-  <si>
     <t>Check whether external links work</t>
   </si>
   <si>
@@ -258,9 +246,6 @@
   </si>
   <si>
     <t>References_test.java</t>
-  </si>
-  <si>
-    <t>References</t>
   </si>
   <si>
     <t>Check whether references are displayed</t>
@@ -281,9 +266,6 @@
     <t>Images_Test.java</t>
   </si>
   <si>
-    <t>Images</t>
-  </si>
-  <si>
     <t>Check whether article images are displayed</t>
   </si>
   <si>
@@ -300,9 +282,6 @@
   </si>
   <si>
     <t>HomeNavigationTest.java</t>
-  </si>
-  <si>
-    <t>Home Page Navigation</t>
   </si>
   <si>
     <t>Check whether Wikipedia home page opens</t>
@@ -385,9 +364,6 @@
     <t>Back_Button_Test.java</t>
   </si>
   <si>
-    <t>Back Button</t>
-  </si>
-  <si>
     <t>Check whether browser back button works</t>
   </si>
   <si>
@@ -417,9 +393,6 @@
     <t>Forward Button</t>
   </si>
   <si>
-    <t>Check whether browser forward button works</t>
-  </si>
-  <si>
     <t>Go back and then use Forward button</t>
   </si>
   <si>
@@ -435,6 +408,32 @@
 10. find tile and store in variable
 11. now compare both article title varible
 12. if is equal than back button work properly else not working.</t>
+  </si>
+  <si>
+    <t>Check whether page works after refresh</t>
+  </si>
+  <si>
+    <t>Refresh an opened article</t>
+  </si>
+  <si>
+    <t>1.Open CgromeBrower
+2. Got to wikipedia
+3. Search India
+4. Click on search button
+5. Find title ans store in variable title
+6. Refresh the page 
+7. Find title and store in variable title2
+8. Compare both title (title &amp; title2).
+9. if same Than refresh button work properly else not.</t>
+  </si>
+  <si>
+    <t>Refresh_Button_Test.java</t>
+  </si>
+  <si>
+    <t>Article Testing</t>
+  </si>
+  <si>
+    <t>Navigation Testing</t>
   </si>
 </sst>
 </file>
@@ -959,23 +958,23 @@
       <c r="B7" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D7" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="E7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="F7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="F7" s="5" t="s">
+      <c r="G7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="H7" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="H7" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="108">
@@ -983,25 +982,25 @@
         <v>2</v>
       </c>
       <c r="B8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D8" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>13</v>
-      </c>
-      <c r="D8" s="4" t="s">
+      <c r="E8" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E8" s="4" t="s">
+      <c r="F8" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="F8" s="5" t="s">
-        <v>22</v>
-      </c>
       <c r="G8" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="90">
@@ -1009,25 +1008,25 @@
         <v>3</v>
       </c>
       <c r="B9" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C9" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="D9" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="E9" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="F9" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="F9" s="5" t="s">
-        <v>27</v>
-      </c>
       <c r="G9" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H9" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="H9" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="132" customHeight="1">
@@ -1035,25 +1034,25 @@
         <v>4</v>
       </c>
       <c r="B10" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D10" s="4" t="s">
         <v>28</v>
       </c>
-      <c r="C10" s="4" t="s">
+      <c r="E10" s="4" t="s">
         <v>29</v>
       </c>
-      <c r="D10" s="4" t="s">
+      <c r="F10" s="5" t="s">
         <v>30</v>
       </c>
-      <c r="E10" s="4" t="s">
+      <c r="G10" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H10" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>32</v>
-      </c>
-      <c r="G10" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="H10" s="4" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="162">
@@ -1061,25 +1060,25 @@
         <v>5</v>
       </c>
       <c r="B11" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C11" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D11" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="E11" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>29</v>
-      </c>
-      <c r="D11" s="4" t="s">
+      <c r="F11" s="5" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>37</v>
-      </c>
       <c r="G11" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H11" s="4" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="162">
@@ -1087,25 +1086,25 @@
         <v>6</v>
       </c>
       <c r="B12" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" s="4" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="C12" s="4" t="s">
+      <c r="F12" s="5" t="s">
         <v>39</v>
       </c>
-      <c r="D12" s="4" t="s">
-        <v>40</v>
-      </c>
-      <c r="E12" s="4" t="s">
-        <v>41</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>42</v>
-      </c>
       <c r="G12" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H12" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="H12" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="108">
@@ -1113,25 +1112,25 @@
         <v>7</v>
       </c>
       <c r="B13" s="4" t="s">
+        <v>40</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>77</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>42</v>
+      </c>
+      <c r="F13" s="5" t="s">
         <v>43</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>44</v>
-      </c>
-      <c r="D13" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="E13" s="4" t="s">
-        <v>46</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>47</v>
-      </c>
       <c r="G13" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H13" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="H13" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="144">
@@ -1139,25 +1138,25 @@
         <v>8</v>
       </c>
       <c r="B14" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>49</v>
+        <v>44</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>77</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="E14" s="4" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="G14" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H14" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="H14" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="15" spans="1:8" ht="126">
@@ -1165,25 +1164,25 @@
         <v>9</v>
       </c>
       <c r="B15" s="4" t="s">
-        <v>53</v>
-      </c>
-      <c r="C15" s="4" t="s">
-        <v>54</v>
+        <v>48</v>
+      </c>
+      <c r="C15" s="7" t="s">
+        <v>77</v>
       </c>
       <c r="D15" s="4" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E15" s="4" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="F15" s="5" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="G15" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="H15" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="H15" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="126">
@@ -1191,25 +1190,25 @@
         <v>10</v>
       </c>
       <c r="B16" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="C16" s="7" t="s">
-        <v>59</v>
+        <v>78</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>60</v>
+        <v>53</v>
       </c>
       <c r="E16" s="7" t="s">
-        <v>61</v>
+        <v>54</v>
       </c>
       <c r="F16" s="8" t="s">
-        <v>62</v>
+        <v>55</v>
       </c>
       <c r="G16" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H16" s="4" t="s">
         <v>17</v>
-      </c>
-      <c r="H16" s="4" t="s">
-        <v>18</v>
       </c>
     </row>
     <row r="17" spans="1:8" ht="234">
@@ -1217,25 +1216,25 @@
         <v>11</v>
       </c>
       <c r="B17" s="7" t="s">
-        <v>71</v>
+        <v>64</v>
       </c>
       <c r="C17" s="7" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="D17" s="7" t="s">
-        <v>73</v>
+        <v>65</v>
       </c>
       <c r="E17" s="7" t="s">
-        <v>74</v>
+        <v>66</v>
       </c>
       <c r="F17" s="8" t="s">
-        <v>76</v>
+        <v>68</v>
       </c>
       <c r="G17" s="7" t="s">
-        <v>75</v>
+        <v>67</v>
       </c>
       <c r="H17" s="4" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="252">
@@ -1243,36 +1242,52 @@
         <v>12</v>
       </c>
       <c r="B18" s="7" t="s">
-        <v>77</v>
+        <v>69</v>
       </c>
       <c r="C18" s="7" t="s">
         <v>78</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>79</v>
+        <v>70</v>
       </c>
       <c r="E18" s="7" t="s">
-        <v>80</v>
+        <v>71</v>
       </c>
       <c r="F18" s="8" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="G18" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H18" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="H18" s="7" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" ht="18">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
+    </row>
+    <row r="19" spans="1:8" s="7" customFormat="1" ht="198">
+      <c r="A19" s="7">
+        <v>13</v>
+      </c>
+      <c r="B19" s="7" t="s">
+        <v>76</v>
+      </c>
+      <c r="C19" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D19" s="7" t="s">
+        <v>73</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>74</v>
+      </c>
+      <c r="F19" s="8" t="s">
+        <v>75</v>
+      </c>
+      <c r="G19" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="20" spans="1:8" ht="18">
       <c r="A20" s="7"/>
@@ -1280,7 +1295,7 @@
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
       <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
+      <c r="F20" s="8"/>
       <c r="G20" s="7"/>
       <c r="H20" s="7"/>
     </row>
@@ -1290,7 +1305,7 @@
       <c r="C21" s="7"/>
       <c r="D21" s="7"/>
       <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
+      <c r="F21" s="8"/>
       <c r="G21" s="7"/>
       <c r="H21" s="7"/>
     </row>
@@ -2464,7 +2479,7 @@
       <c r="D4" s="17"/>
       <c r="E4" s="17"/>
       <c r="F4" s="17" t="s">
-        <v>63</v>
+        <v>56</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
@@ -2499,7 +2514,7 @@
         <v>9</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="H6" s="1" t="s">
         <v>11</v>
@@ -2510,13 +2525,13 @@
         <v>1</v>
       </c>
       <c r="B7" t="s">
-        <v>65</v>
+        <v>58</v>
       </c>
       <c r="C7" t="s">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="D7" t="s">
-        <v>67</v>
+        <v>60</v>
       </c>
     </row>
     <row r="8" spans="1:8" ht="117.6" customHeight="1"/>
@@ -2590,7 +2605,7 @@
       <c r="D4" s="17"/>
       <c r="E4" s="17"/>
       <c r="F4" s="17" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
@@ -2625,10 +2640,10 @@
         <v>9</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>
@@ -2700,7 +2715,7 @@
       <c r="D4" s="17"/>
       <c r="E4" s="17"/>
       <c r="F4" s="17" t="s">
-        <v>68</v>
+        <v>61</v>
       </c>
       <c r="G4" s="17"/>
       <c r="H4" s="17"/>
@@ -2735,10 +2750,10 @@
         <v>9</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>70</v>
+        <v>63</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Implement Multiple Article Navigation testing in file src/Navigation_Testing/Multiple_Article_Navigation_Test.java , test is pass, && Add multiple Article Navigation test status column in  wikipedia-Testing-ExcelSheet.xlsx file ,Status of the test is pass.
</commit_message>
<xml_diff>
--- a/wikipedia-Testing-ExcelSheet.xlsx
+++ b/wikipedia-Testing-ExcelSheet.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECT\wikipedia_testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B524CD51-B1C7-45C7-AF58-783C80DC38E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5C50805-45DC-4CF3-8B83-E78772352977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="79">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="83">
   <si>
     <t>Wikipedia Search &amp; Reader UI</t>
   </si>
@@ -434,6 +434,29 @@
   </si>
   <si>
     <t>Navigation Testing</t>
+  </si>
+  <si>
+    <t>Multiple_Article_Navigation_Test</t>
+  </si>
+  <si>
+    <t>Check navigation between multiple articles</t>
+  </si>
+  <si>
+    <t>Open multiple articles one by one</t>
+  </si>
+  <si>
+    <t>1. open chromeDriver
+2. Go to wikipedia
+3. Search India
+4. Click on Search button
+5. Find title , store title and ckeck title is India or not…
+6. Now search youtube
+7. click on Search button
+8. Find title,store title and check title is youtube or not
+9. Now search Amazon
+10. Click on Search button
+11. Find title,store title and check title is amazon or not
+12. Now final check all the title are same or not if yes than test pass , else test fail.</t>
   </si>
 </sst>
 </file>
@@ -1289,15 +1312,31 @@
         <v>17</v>
       </c>
     </row>
-    <row r="20" spans="1:8" ht="18">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="7"/>
-      <c r="H20" s="7"/>
+    <row r="20" spans="1:8" s="7" customFormat="1" ht="306">
+      <c r="A20" s="7">
+        <v>14</v>
+      </c>
+      <c r="B20" s="7" t="s">
+        <v>79</v>
+      </c>
+      <c r="C20" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" s="7" t="s">
+        <v>80</v>
+      </c>
+      <c r="E20" s="7" t="s">
+        <v>81</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>82</v>
+      </c>
+      <c r="G20" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H20" s="7" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="21" spans="1:8" ht="18">
       <c r="A21" s="7"/>

</xml_diff>

<commit_message>
- Converted the project to Apache Maven project - Set up standard Maven structure: src/main/java and src/test/java - Moved all test cases into src/test/java - Moved Xpath.properties into src/test/resources
</commit_message>
<xml_diff>
--- a/wikipedia-Testing-ExcelSheet.xlsx
+++ b/wikipedia-Testing-ExcelSheet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\PROJECT\wikipedia_testing\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5C50805-45DC-4CF3-8B83-E78772352977}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4CFD59CC-5CD2-4CA8-823B-2BBD480A652A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="13776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Akash" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="149" uniqueCount="83">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="155" uniqueCount="86">
   <si>
     <t>Wikipedia Search &amp; Reader UI</t>
   </si>
@@ -457,6 +457,15 @@
 10. Click on Search button
 11. Find title,store title and check title is amazon or not
 12. Now final check all the title are same or not if yes than test pass , else test fail.</t>
+  </si>
+  <si>
+    <t>Page_Scrolling_Test.java</t>
+  </si>
+  <si>
+    <t>Check whether article page can be scrolled</t>
+  </si>
+  <si>
+    <t>Scroll from top to bottom of article</t>
   </si>
 </sst>
 </file>
@@ -1338,15 +1347,29 @@
         <v>17</v>
       </c>
     </row>
-    <row r="21" spans="1:8" ht="18">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
+    <row r="21" spans="1:8" ht="36">
+      <c r="A21" s="7">
+        <v>15</v>
+      </c>
+      <c r="B21" s="7" t="s">
+        <v>83</v>
+      </c>
+      <c r="C21" s="7" t="s">
+        <v>78</v>
+      </c>
+      <c r="D21" s="7" t="s">
+        <v>84</v>
+      </c>
+      <c r="E21" s="7" t="s">
+        <v>85</v>
+      </c>
       <c r="F21" s="8"/>
-      <c r="G21" s="7"/>
-      <c r="H21" s="7"/>
+      <c r="G21" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="22" spans="1:8" ht="18">
       <c r="A22" s="7"/>

</xml_diff>